<commit_message>
scrp ini data analysis
</commit_message>
<xml_diff>
--- a/barrier-land-title/data/land-title.xlsx
+++ b/barrier-land-title/data/land-title.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viser\Desktop\BARRIERS TO LAND TITLING IN PALO LEYTE_2026\FINAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viser\OneDrive\Dokumen\Github repository\data-consultation-2026\barrier-land-title\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4765172C-9229-4ED0-8E1A-E0DE5C3A700B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3071A056-FFB1-47AE-AB7A-288AC36D4598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="22" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -29,8 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
@@ -1675,7 +1673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1708,7 +1706,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15612,7 +15609,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FE808742-FC19-4B48-95BF-EF84F6EEE75F}" name="PivotTable1" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FE808742-FC19-4B48-95BF-EF84F6EEE75F}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="75">
     <pivotField dataField="1" showAll="0"/>
@@ -15990,7 +15987,7 @@
       <c r="A4" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="24">
+      <c r="B4">
         <v>26</v>
       </c>
     </row>
@@ -15998,7 +15995,7 @@
       <c r="A5" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5">
         <v>33</v>
       </c>
     </row>
@@ -16006,7 +16003,7 @@
       <c r="A6" s="23" t="s">
         <v>196</v>
       </c>
-      <c r="B6" s="24">
+      <c r="B6">
         <v>25</v>
       </c>
     </row>
@@ -16014,7 +16011,7 @@
       <c r="A7" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7">
         <v>31</v>
       </c>
     </row>
@@ -16022,7 +16019,7 @@
       <c r="A8" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="B8" s="24">
+      <c r="B8">
         <v>27</v>
       </c>
     </row>
@@ -16030,7 +16027,7 @@
       <c r="A9" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9">
         <v>35</v>
       </c>
     </row>
@@ -16038,7 +16035,7 @@
       <c r="A10" s="23" t="s">
         <v>502</v>
       </c>
-      <c r="B10" s="24">
+      <c r="B10">
         <v>177</v>
       </c>
     </row>

</xml_diff>